<commit_message>
Enforce estimate applicability gates
</commit_message>
<xml_diff>
--- a/prepare-local-cost-estimate/assets/lsr-rim-template.xlsx
+++ b/prepare-local-cost-estimate/assets/lsr-rim-template.xlsx
@@ -2321,7 +2321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2338,8 +2338,8 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
@@ -2347,8 +2347,11 @@
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="42" customWidth="1" min="24" max="24"/>
-    <col width="42" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="42" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -2419,60 +2422,75 @@
       </c>
       <c r="N1" s="10" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Статус применимости нормы</t>
         </is>
       </c>
       <c r="O1" s="10" t="inlineStr">
         <is>
+          <t>Матрица сопоставления</t>
+        </is>
+      </c>
+      <c r="P1" s="10" t="inlineStr">
+        <is>
+          <t>Границы учтённых работ</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>Статус расчёта</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
           <t>Ответ / уточнение пользователя</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="S1" s="10" t="inlineStr">
         <is>
           <t>Решение после ответа</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="T1" s="10" t="inlineStr">
         <is>
           <t>price_kind</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="U1" s="10" t="inlineStr">
         <is>
           <t>price_base</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="V1" s="10" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="T1" s="10" t="inlineStr">
+      <c r="W1" s="10" t="inlineStr">
         <is>
           <t>Группа однородных ресурсов</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="X1" s="10" t="inlineStr">
         <is>
           <t>resolved_price</t>
         </is>
       </c>
-      <c r="V1" s="10" t="inlineStr">
+      <c r="Y1" s="10" t="inlineStr">
         <is>
           <t>zone_id</t>
         </is>
       </c>
-      <c r="W1" s="10" t="inlineStr">
+      <c r="Z1" s="10" t="inlineStr">
         <is>
           <t>period_id</t>
         </is>
       </c>
-      <c r="X1" s="10" t="inlineStr">
+      <c r="AA1" s="10" t="inlineStr">
         <is>
           <t>dataset / source row</t>
         </is>
       </c>
-      <c r="Y1" s="10" t="inlineStr">
+      <c r="AB1" s="10" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>

</xml_diff>